<commit_message>
Record phase 3 decisions; add the updated rate card (EUR retail and commission, EGP operator amounts)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LdY5dQmdpbpwvFGXgFTg1y
</commit_message>
<xml_diff>
--- a/docs/model/sawa-rate-card.xlsx
+++ b/docs/model/sawa-rate-card.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="204" uniqueCount="121">
   <si>
     <t xml:space="preserve">Sawa rate card</t>
   </si>
@@ -41,7 +41,7 @@
     <t xml:space="preserve">Yellow cells with blue text are inputs. Everything else is calculated: don't overwrite it.</t>
   </si>
   <si>
-    <t xml:space="preserve">Amounts are in the currency set on the Assumptions sheet.</t>
+    <t xml:space="preserve">Currencies: the retail price and agency commission are in EUR; every operator amount is in EGP. Margins are shown in EUR, converted with the exchange rate on the Assumptions sheet.</t>
   </si>
   <si>
     <t xml:space="preserve">The first row on each product sheet (shaded, marked EXAMPLE) uses illustrative numbers to show the formulas working. Delete or overwrite it once real rows are filled.</t>
@@ -89,13 +89,28 @@
     <t xml:space="preserve">Note</t>
   </si>
   <si>
-    <t xml:space="preserve">Currency</t>
-  </si>
-  <si>
-    <t xml:space="preserve">USD</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Replace with the currency you agree with operators (clause 9.4).</t>
+    <t xml:space="preserve">Traveller currency (retail price, agency commission)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EUR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Travellers pay in EUR; agency commission is set per seat in EUR.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Operator currency (all operator amounts)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EGP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Departure fees, per-traveller amounts, rooms and cabins are paid to operators in EGP.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Exchange rate: EGP per 1 EUR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Placeholder. Replace with the current rate; margins below convert operator costs to EUR with it.</t>
   </si>
   <si>
     <t xml:space="preserve">Payment processing fee (% of retail)</t>
@@ -158,13 +173,13 @@
     <t xml:space="preserve">Agency commission per seat</t>
   </si>
   <si>
-    <t xml:space="preserve">Sawa margin A: 4 direct</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sawa margin B: 8 (5 direct, 3 agency)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sawa margin C: 12 (6 direct, 6 agency)</t>
+    <t xml:space="preserve">Sawa margin A (EUR): 4 direct</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sawa margin B (EUR): 8 (5 direct, 3 agency)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sawa margin C (EUR): 12 (6 direct, 6 agency)</t>
   </si>
   <si>
     <t xml:space="preserve">Loss at 4?</t>
@@ -308,13 +323,13 @@
     <t xml:space="preserve">Room/cabin per trip: single (per room)</t>
   </si>
   <si>
-    <t xml:space="preserve">Sawa margin A: 4 direct, 2 twin rooms</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sawa margin B: 4 direct, 1 twin + 2 singles</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cost of single promise</t>
+    <t xml:space="preserve">Sawa margin A (EUR): 4 direct, 2 twin rooms</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sawa margin B (EUR): 4 direct, 1 twin + 2 singles</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cost of single promise (EUR)</t>
   </si>
   <si>
     <t xml:space="preserve">Cruise</t>
@@ -875,7 +890,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
         <v>5</v>
       </c>
@@ -960,7 +975,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40"/>
@@ -999,55 +1014,77 @@
       <c r="A5" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="B5" s="8" t="n">
-        <v>0.03</v>
+      <c r="B5" s="7" t="s">
+        <v>25</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B6" s="7" t="n">
-        <v>5</v>
+        <v>55</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="B7" s="7" t="n">
-        <v>3</v>
+        <v>29</v>
+      </c>
+      <c r="B7" s="8" t="n">
+        <v>0.03</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B8" s="7" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B9" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="B10" s="7" t="n">
         <v>6</v>
       </c>
-      <c r="C9" s="6" t="s">
-        <v>30</v>
+      <c r="C10" s="6" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="B11" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -1082,103 +1119,103 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="9" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="F3" s="9" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="G3" s="9" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="H3" s="9" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="I3" s="9" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="J3" s="9" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="K3" s="9" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="L3" s="9" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="M3" s="9" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="N3" s="9" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="O3" s="9" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="P3" s="9" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="10" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="F4" s="11" t="n">
         <v>95</v>
       </c>
       <c r="G4" s="11" t="n">
-        <v>40</v>
+        <v>2200</v>
       </c>
       <c r="H4" s="11" t="n">
-        <v>150</v>
+        <v>8250</v>
       </c>
       <c r="I4" s="11" t="n">
-        <v>200</v>
+        <v>11000</v>
       </c>
       <c r="J4" s="11" t="n">
-        <v>250</v>
+        <v>13750</v>
       </c>
       <c r="K4" s="11" t="n">
         <v>12</v>
       </c>
       <c r="L4" s="12" t="n">
-        <f aca="false">IF(F4="","",4*F4-(4*G4+H4)-4*F4*Assumptions!$B$5)</f>
+        <f aca="false">IF(F4="","",4*F4-(4*G4+H4)/Assumptions!$B$6-4*F4*Assumptions!$B$7)</f>
         <v>58.6</v>
       </c>
       <c r="M4" s="12" t="n">
-        <f aca="false">IF(F4="","",(Assumptions!$B$6+Assumptions!$B$7)*F4-((Assumptions!$B$6+Assumptions!$B$7)*G4+I4)-Assumptions!$B$7*K4-(Assumptions!$B$6+Assumptions!$B$7)*F4*Assumptions!$B$5)</f>
+        <f aca="false">IF(F4="","",(Assumptions!$B$8+Assumptions!$B$9)*F4-((Assumptions!$B$8+Assumptions!$B$9)*G4+I4)/Assumptions!$B$6-Assumptions!$B$9*K4-(Assumptions!$B$8+Assumptions!$B$9)*F4*Assumptions!$B$7)</f>
         <v>181.2</v>
       </c>
       <c r="N4" s="12" t="n">
-        <f aca="false">IF(F4="","",(Assumptions!$B$8+Assumptions!$B$9)*F4-((Assumptions!$B$8+Assumptions!$B$9)*G4+J4)-Assumptions!$B$9*K4-(Assumptions!$B$8+Assumptions!$B$9)*F4*Assumptions!$B$5)</f>
+        <f aca="false">IF(F4="","",(Assumptions!$B$10+Assumptions!$B$11)*F4-((Assumptions!$B$10+Assumptions!$B$11)*G4+J4)/Assumptions!$B$6-Assumptions!$B$11*K4-(Assumptions!$B$10+Assumptions!$B$11)*F4*Assumptions!$B$7)</f>
         <v>303.8</v>
       </c>
       <c r="O4" s="12" t="str">
@@ -1186,7 +1223,7 @@
         <v>OK</v>
       </c>
       <c r="P4" s="10" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1194,16 +1231,16 @@
         <v>1</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="C5" s="13" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="D5" s="13" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="E5" s="13" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="F5" s="11"/>
       <c r="G5" s="11"/>
@@ -1212,15 +1249,15 @@
       <c r="J5" s="11"/>
       <c r="K5" s="11"/>
       <c r="L5" s="14" t="str">
-        <f aca="false">IF(F5="","",4*F5-(4*G5+H5)-4*F5*Assumptions!$B$5)</f>
+        <f aca="false">IF(F5="","",4*F5-(4*G5+H5)/Assumptions!$B$6-4*F5*Assumptions!$B$7)</f>
         <v/>
       </c>
       <c r="M5" s="14" t="str">
-        <f aca="false">IF(F5="","",(Assumptions!$B$6+Assumptions!$B$7)*F5-((Assumptions!$B$6+Assumptions!$B$7)*G5+I5)-Assumptions!$B$7*K5-(Assumptions!$B$6+Assumptions!$B$7)*F5*Assumptions!$B$5)</f>
+        <f aca="false">IF(F5="","",(Assumptions!$B$8+Assumptions!$B$9)*F5-((Assumptions!$B$8+Assumptions!$B$9)*G5+I5)/Assumptions!$B$6-Assumptions!$B$9*K5-(Assumptions!$B$8+Assumptions!$B$9)*F5*Assumptions!$B$7)</f>
         <v/>
       </c>
       <c r="N5" s="14" t="str">
-        <f aca="false">IF(F5="","",(Assumptions!$B$8+Assumptions!$B$9)*F5-((Assumptions!$B$8+Assumptions!$B$9)*G5+J5)-Assumptions!$B$9*K5-(Assumptions!$B$8+Assumptions!$B$9)*F5*Assumptions!$B$5)</f>
+        <f aca="false">IF(F5="","",(Assumptions!$B$10+Assumptions!$B$11)*F5-((Assumptions!$B$10+Assumptions!$B$11)*G5+J5)/Assumptions!$B$6-Assumptions!$B$11*K5-(Assumptions!$B$10+Assumptions!$B$11)*F5*Assumptions!$B$7)</f>
         <v/>
       </c>
       <c r="O5" s="14" t="str">
@@ -1234,16 +1271,16 @@
         <v>2</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="D6" s="13" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="E6" s="13" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="F6" s="11"/>
       <c r="G6" s="11"/>
@@ -1252,15 +1289,15 @@
       <c r="J6" s="11"/>
       <c r="K6" s="11"/>
       <c r="L6" s="14" t="str">
-        <f aca="false">IF(F6="","",4*F6-(4*G6+H6)-4*F6*Assumptions!$B$5)</f>
+        <f aca="false">IF(F6="","",4*F6-(4*G6+H6)/Assumptions!$B$6-4*F6*Assumptions!$B$7)</f>
         <v/>
       </c>
       <c r="M6" s="14" t="str">
-        <f aca="false">IF(F6="","",(Assumptions!$B$6+Assumptions!$B$7)*F6-((Assumptions!$B$6+Assumptions!$B$7)*G6+I6)-Assumptions!$B$7*K6-(Assumptions!$B$6+Assumptions!$B$7)*F6*Assumptions!$B$5)</f>
+        <f aca="false">IF(F6="","",(Assumptions!$B$8+Assumptions!$B$9)*F6-((Assumptions!$B$8+Assumptions!$B$9)*G6+I6)/Assumptions!$B$6-Assumptions!$B$9*K6-(Assumptions!$B$8+Assumptions!$B$9)*F6*Assumptions!$B$7)</f>
         <v/>
       </c>
       <c r="N6" s="14" t="str">
-        <f aca="false">IF(F6="","",(Assumptions!$B$8+Assumptions!$B$9)*F6-((Assumptions!$B$8+Assumptions!$B$9)*G6+J6)-Assumptions!$B$9*K6-(Assumptions!$B$8+Assumptions!$B$9)*F6*Assumptions!$B$5)</f>
+        <f aca="false">IF(F6="","",(Assumptions!$B$10+Assumptions!$B$11)*F6-((Assumptions!$B$10+Assumptions!$B$11)*G6+J6)/Assumptions!$B$6-Assumptions!$B$11*K6-(Assumptions!$B$10+Assumptions!$B$11)*F6*Assumptions!$B$7)</f>
         <v/>
       </c>
       <c r="O6" s="14" t="str">
@@ -1268,7 +1305,7 @@
         <v/>
       </c>
       <c r="P6" s="13" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1276,16 +1313,16 @@
         <v>3</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="C7" s="13" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="D7" s="13" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="E7" s="13" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="F7" s="11"/>
       <c r="G7" s="11"/>
@@ -1294,15 +1331,15 @@
       <c r="J7" s="11"/>
       <c r="K7" s="11"/>
       <c r="L7" s="14" t="str">
-        <f aca="false">IF(F7="","",4*F7-(4*G7+H7)-4*F7*Assumptions!$B$5)</f>
+        <f aca="false">IF(F7="","",4*F7-(4*G7+H7)/Assumptions!$B$6-4*F7*Assumptions!$B$7)</f>
         <v/>
       </c>
       <c r="M7" s="14" t="str">
-        <f aca="false">IF(F7="","",(Assumptions!$B$6+Assumptions!$B$7)*F7-((Assumptions!$B$6+Assumptions!$B$7)*G7+I7)-Assumptions!$B$7*K7-(Assumptions!$B$6+Assumptions!$B$7)*F7*Assumptions!$B$5)</f>
+        <f aca="false">IF(F7="","",(Assumptions!$B$8+Assumptions!$B$9)*F7-((Assumptions!$B$8+Assumptions!$B$9)*G7+I7)/Assumptions!$B$6-Assumptions!$B$9*K7-(Assumptions!$B$8+Assumptions!$B$9)*F7*Assumptions!$B$7)</f>
         <v/>
       </c>
       <c r="N7" s="14" t="str">
-        <f aca="false">IF(F7="","",(Assumptions!$B$8+Assumptions!$B$9)*F7-((Assumptions!$B$8+Assumptions!$B$9)*G7+J7)-Assumptions!$B$9*K7-(Assumptions!$B$8+Assumptions!$B$9)*F7*Assumptions!$B$5)</f>
+        <f aca="false">IF(F7="","",(Assumptions!$B$10+Assumptions!$B$11)*F7-((Assumptions!$B$10+Assumptions!$B$11)*G7+J7)/Assumptions!$B$6-Assumptions!$B$11*K7-(Assumptions!$B$10+Assumptions!$B$11)*F7*Assumptions!$B$7)</f>
         <v/>
       </c>
       <c r="O7" s="14" t="str">
@@ -1310,7 +1347,7 @@
         <v/>
       </c>
       <c r="P7" s="13" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1318,16 +1355,16 @@
         <v>4</v>
       </c>
       <c r="B8" s="13" t="s">
+        <v>66</v>
+      </c>
+      <c r="C8" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="D8" s="13" t="s">
         <v>61</v>
       </c>
-      <c r="C8" s="13" t="s">
-        <v>51</v>
-      </c>
-      <c r="D8" s="13" t="s">
-        <v>56</v>
-      </c>
       <c r="E8" s="13" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="F8" s="11"/>
       <c r="G8" s="11"/>
@@ -1336,15 +1373,15 @@
       <c r="J8" s="11"/>
       <c r="K8" s="11"/>
       <c r="L8" s="14" t="str">
-        <f aca="false">IF(F8="","",4*F8-(4*G8+H8)-4*F8*Assumptions!$B$5)</f>
+        <f aca="false">IF(F8="","",4*F8-(4*G8+H8)/Assumptions!$B$6-4*F8*Assumptions!$B$7)</f>
         <v/>
       </c>
       <c r="M8" s="14" t="str">
-        <f aca="false">IF(F8="","",(Assumptions!$B$6+Assumptions!$B$7)*F8-((Assumptions!$B$6+Assumptions!$B$7)*G8+I8)-Assumptions!$B$7*K8-(Assumptions!$B$6+Assumptions!$B$7)*F8*Assumptions!$B$5)</f>
+        <f aca="false">IF(F8="","",(Assumptions!$B$8+Assumptions!$B$9)*F8-((Assumptions!$B$8+Assumptions!$B$9)*G8+I8)/Assumptions!$B$6-Assumptions!$B$9*K8-(Assumptions!$B$8+Assumptions!$B$9)*F8*Assumptions!$B$7)</f>
         <v/>
       </c>
       <c r="N8" s="14" t="str">
-        <f aca="false">IF(F8="","",(Assumptions!$B$8+Assumptions!$B$9)*F8-((Assumptions!$B$8+Assumptions!$B$9)*G8+J8)-Assumptions!$B$9*K8-(Assumptions!$B$8+Assumptions!$B$9)*F8*Assumptions!$B$5)</f>
+        <f aca="false">IF(F8="","",(Assumptions!$B$10+Assumptions!$B$11)*F8-((Assumptions!$B$10+Assumptions!$B$11)*G8+J8)/Assumptions!$B$6-Assumptions!$B$11*K8-(Assumptions!$B$10+Assumptions!$B$11)*F8*Assumptions!$B$7)</f>
         <v/>
       </c>
       <c r="O8" s="14" t="str">
@@ -1358,16 +1395,16 @@
         <v>5</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="D9" s="13" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="E9" s="13" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="F9" s="11"/>
       <c r="G9" s="11"/>
@@ -1376,15 +1413,15 @@
       <c r="J9" s="11"/>
       <c r="K9" s="11"/>
       <c r="L9" s="14" t="str">
-        <f aca="false">IF(F9="","",4*F9-(4*G9+H9)-4*F9*Assumptions!$B$5)</f>
+        <f aca="false">IF(F9="","",4*F9-(4*G9+H9)/Assumptions!$B$6-4*F9*Assumptions!$B$7)</f>
         <v/>
       </c>
       <c r="M9" s="14" t="str">
-        <f aca="false">IF(F9="","",(Assumptions!$B$6+Assumptions!$B$7)*F9-((Assumptions!$B$6+Assumptions!$B$7)*G9+I9)-Assumptions!$B$7*K9-(Assumptions!$B$6+Assumptions!$B$7)*F9*Assumptions!$B$5)</f>
+        <f aca="false">IF(F9="","",(Assumptions!$B$8+Assumptions!$B$9)*F9-((Assumptions!$B$8+Assumptions!$B$9)*G9+I9)/Assumptions!$B$6-Assumptions!$B$9*K9-(Assumptions!$B$8+Assumptions!$B$9)*F9*Assumptions!$B$7)</f>
         <v/>
       </c>
       <c r="N9" s="14" t="str">
-        <f aca="false">IF(F9="","",(Assumptions!$B$8+Assumptions!$B$9)*F9-((Assumptions!$B$8+Assumptions!$B$9)*G9+J9)-Assumptions!$B$9*K9-(Assumptions!$B$8+Assumptions!$B$9)*F9*Assumptions!$B$5)</f>
+        <f aca="false">IF(F9="","",(Assumptions!$B$10+Assumptions!$B$11)*F9-((Assumptions!$B$10+Assumptions!$B$11)*G9+J9)/Assumptions!$B$6-Assumptions!$B$11*K9-(Assumptions!$B$10+Assumptions!$B$11)*F9*Assumptions!$B$7)</f>
         <v/>
       </c>
       <c r="O9" s="14" t="str">
@@ -1398,16 +1435,16 @@
         <v>6</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="C10" s="13" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="D10" s="13" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="E10" s="13" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="F10" s="11"/>
       <c r="G10" s="11"/>
@@ -1416,15 +1453,15 @@
       <c r="J10" s="11"/>
       <c r="K10" s="11"/>
       <c r="L10" s="14" t="str">
-        <f aca="false">IF(F10="","",4*F10-(4*G10+H10)-4*F10*Assumptions!$B$5)</f>
+        <f aca="false">IF(F10="","",4*F10-(4*G10+H10)/Assumptions!$B$6-4*F10*Assumptions!$B$7)</f>
         <v/>
       </c>
       <c r="M10" s="14" t="str">
-        <f aca="false">IF(F10="","",(Assumptions!$B$6+Assumptions!$B$7)*F10-((Assumptions!$B$6+Assumptions!$B$7)*G10+I10)-Assumptions!$B$7*K10-(Assumptions!$B$6+Assumptions!$B$7)*F10*Assumptions!$B$5)</f>
+        <f aca="false">IF(F10="","",(Assumptions!$B$8+Assumptions!$B$9)*F10-((Assumptions!$B$8+Assumptions!$B$9)*G10+I10)/Assumptions!$B$6-Assumptions!$B$9*K10-(Assumptions!$B$8+Assumptions!$B$9)*F10*Assumptions!$B$7)</f>
         <v/>
       </c>
       <c r="N10" s="14" t="str">
-        <f aca="false">IF(F10="","",(Assumptions!$B$8+Assumptions!$B$9)*F10-((Assumptions!$B$8+Assumptions!$B$9)*G10+J10)-Assumptions!$B$9*K10-(Assumptions!$B$8+Assumptions!$B$9)*F10*Assumptions!$B$5)</f>
+        <f aca="false">IF(F10="","",(Assumptions!$B$10+Assumptions!$B$11)*F10-((Assumptions!$B$10+Assumptions!$B$11)*G10+J10)/Assumptions!$B$6-Assumptions!$B$11*K10-(Assumptions!$B$10+Assumptions!$B$11)*F10*Assumptions!$B$7)</f>
         <v/>
       </c>
       <c r="O10" s="14" t="str">
@@ -1438,16 +1475,16 @@
         <v>7</v>
       </c>
       <c r="B11" s="13" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="C11" s="13" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="D11" s="13" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="E11" s="13" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="F11" s="11"/>
       <c r="G11" s="11"/>
@@ -1456,15 +1493,15 @@
       <c r="J11" s="11"/>
       <c r="K11" s="11"/>
       <c r="L11" s="14" t="str">
-        <f aca="false">IF(F11="","",4*F11-(4*G11+H11)-4*F11*Assumptions!$B$5)</f>
+        <f aca="false">IF(F11="","",4*F11-(4*G11+H11)/Assumptions!$B$6-4*F11*Assumptions!$B$7)</f>
         <v/>
       </c>
       <c r="M11" s="14" t="str">
-        <f aca="false">IF(F11="","",(Assumptions!$B$6+Assumptions!$B$7)*F11-((Assumptions!$B$6+Assumptions!$B$7)*G11+I11)-Assumptions!$B$7*K11-(Assumptions!$B$6+Assumptions!$B$7)*F11*Assumptions!$B$5)</f>
+        <f aca="false">IF(F11="","",(Assumptions!$B$8+Assumptions!$B$9)*F11-((Assumptions!$B$8+Assumptions!$B$9)*G11+I11)/Assumptions!$B$6-Assumptions!$B$9*K11-(Assumptions!$B$8+Assumptions!$B$9)*F11*Assumptions!$B$7)</f>
         <v/>
       </c>
       <c r="N11" s="14" t="str">
-        <f aca="false">IF(F11="","",(Assumptions!$B$8+Assumptions!$B$9)*F11-((Assumptions!$B$8+Assumptions!$B$9)*G11+J11)-Assumptions!$B$9*K11-(Assumptions!$B$8+Assumptions!$B$9)*F11*Assumptions!$B$5)</f>
+        <f aca="false">IF(F11="","",(Assumptions!$B$10+Assumptions!$B$11)*F11-((Assumptions!$B$10+Assumptions!$B$11)*G11+J11)/Assumptions!$B$6-Assumptions!$B$11*K11-(Assumptions!$B$10+Assumptions!$B$11)*F11*Assumptions!$B$7)</f>
         <v/>
       </c>
       <c r="O11" s="14" t="str">
@@ -1472,7 +1509,7 @@
         <v/>
       </c>
       <c r="P11" s="13" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1480,16 +1517,16 @@
         <v>8</v>
       </c>
       <c r="B12" s="13" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="C12" s="13" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="D12" s="13" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="E12" s="13" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="F12" s="11"/>
       <c r="G12" s="11"/>
@@ -1498,15 +1535,15 @@
       <c r="J12" s="11"/>
       <c r="K12" s="11"/>
       <c r="L12" s="14" t="str">
-        <f aca="false">IF(F12="","",4*F12-(4*G12+H12)-4*F12*Assumptions!$B$5)</f>
+        <f aca="false">IF(F12="","",4*F12-(4*G12+H12)/Assumptions!$B$6-4*F12*Assumptions!$B$7)</f>
         <v/>
       </c>
       <c r="M12" s="14" t="str">
-        <f aca="false">IF(F12="","",(Assumptions!$B$6+Assumptions!$B$7)*F12-((Assumptions!$B$6+Assumptions!$B$7)*G12+I12)-Assumptions!$B$7*K12-(Assumptions!$B$6+Assumptions!$B$7)*F12*Assumptions!$B$5)</f>
+        <f aca="false">IF(F12="","",(Assumptions!$B$8+Assumptions!$B$9)*F12-((Assumptions!$B$8+Assumptions!$B$9)*G12+I12)/Assumptions!$B$6-Assumptions!$B$9*K12-(Assumptions!$B$8+Assumptions!$B$9)*F12*Assumptions!$B$7)</f>
         <v/>
       </c>
       <c r="N12" s="14" t="str">
-        <f aca="false">IF(F12="","",(Assumptions!$B$8+Assumptions!$B$9)*F12-((Assumptions!$B$8+Assumptions!$B$9)*G12+J12)-Assumptions!$B$9*K12-(Assumptions!$B$8+Assumptions!$B$9)*F12*Assumptions!$B$5)</f>
+        <f aca="false">IF(F12="","",(Assumptions!$B$10+Assumptions!$B$11)*F12-((Assumptions!$B$10+Assumptions!$B$11)*G12+J12)/Assumptions!$B$6-Assumptions!$B$11*K12-(Assumptions!$B$10+Assumptions!$B$11)*F12*Assumptions!$B$7)</f>
         <v/>
       </c>
       <c r="O12" s="14" t="str">
@@ -1514,7 +1551,7 @@
         <v/>
       </c>
       <c r="P12" s="13" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1522,16 +1559,16 @@
         <v>9</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="C13" s="13" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="D13" s="13" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="E13" s="13" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="F13" s="11"/>
       <c r="G13" s="11"/>
@@ -1540,15 +1577,15 @@
       <c r="J13" s="11"/>
       <c r="K13" s="11"/>
       <c r="L13" s="14" t="str">
-        <f aca="false">IF(F13="","",4*F13-(4*G13+H13)-4*F13*Assumptions!$B$5)</f>
+        <f aca="false">IF(F13="","",4*F13-(4*G13+H13)/Assumptions!$B$6-4*F13*Assumptions!$B$7)</f>
         <v/>
       </c>
       <c r="M13" s="14" t="str">
-        <f aca="false">IF(F13="","",(Assumptions!$B$6+Assumptions!$B$7)*F13-((Assumptions!$B$6+Assumptions!$B$7)*G13+I13)-Assumptions!$B$7*K13-(Assumptions!$B$6+Assumptions!$B$7)*F13*Assumptions!$B$5)</f>
+        <f aca="false">IF(F13="","",(Assumptions!$B$8+Assumptions!$B$9)*F13-((Assumptions!$B$8+Assumptions!$B$9)*G13+I13)/Assumptions!$B$6-Assumptions!$B$9*K13-(Assumptions!$B$8+Assumptions!$B$9)*F13*Assumptions!$B$7)</f>
         <v/>
       </c>
       <c r="N13" s="14" t="str">
-        <f aca="false">IF(F13="","",(Assumptions!$B$8+Assumptions!$B$9)*F13-((Assumptions!$B$8+Assumptions!$B$9)*G13+J13)-Assumptions!$B$9*K13-(Assumptions!$B$8+Assumptions!$B$9)*F13*Assumptions!$B$5)</f>
+        <f aca="false">IF(F13="","",(Assumptions!$B$10+Assumptions!$B$11)*F13-((Assumptions!$B$10+Assumptions!$B$11)*G13+J13)/Assumptions!$B$6-Assumptions!$B$11*K13-(Assumptions!$B$10+Assumptions!$B$11)*F13*Assumptions!$B$7)</f>
         <v/>
       </c>
       <c r="O13" s="14" t="str">
@@ -1562,16 +1599,16 @@
         <v>10</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="C14" s="13" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="D14" s="13" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="E14" s="13" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="F14" s="11"/>
       <c r="G14" s="11"/>
@@ -1580,15 +1617,15 @@
       <c r="J14" s="11"/>
       <c r="K14" s="11"/>
       <c r="L14" s="14" t="str">
-        <f aca="false">IF(F14="","",4*F14-(4*G14+H14)-4*F14*Assumptions!$B$5)</f>
+        <f aca="false">IF(F14="","",4*F14-(4*G14+H14)/Assumptions!$B$6-4*F14*Assumptions!$B$7)</f>
         <v/>
       </c>
       <c r="M14" s="14" t="str">
-        <f aca="false">IF(F14="","",(Assumptions!$B$6+Assumptions!$B$7)*F14-((Assumptions!$B$6+Assumptions!$B$7)*G14+I14)-Assumptions!$B$7*K14-(Assumptions!$B$6+Assumptions!$B$7)*F14*Assumptions!$B$5)</f>
+        <f aca="false">IF(F14="","",(Assumptions!$B$8+Assumptions!$B$9)*F14-((Assumptions!$B$8+Assumptions!$B$9)*G14+I14)/Assumptions!$B$6-Assumptions!$B$9*K14-(Assumptions!$B$8+Assumptions!$B$9)*F14*Assumptions!$B$7)</f>
         <v/>
       </c>
       <c r="N14" s="14" t="str">
-        <f aca="false">IF(F14="","",(Assumptions!$B$8+Assumptions!$B$9)*F14-((Assumptions!$B$8+Assumptions!$B$9)*G14+J14)-Assumptions!$B$9*K14-(Assumptions!$B$8+Assumptions!$B$9)*F14*Assumptions!$B$5)</f>
+        <f aca="false">IF(F14="","",(Assumptions!$B$10+Assumptions!$B$11)*F14-((Assumptions!$B$10+Assumptions!$B$11)*G14+J14)/Assumptions!$B$6-Assumptions!$B$11*K14-(Assumptions!$B$10+Assumptions!$B$11)*F14*Assumptions!$B$7)</f>
         <v/>
       </c>
       <c r="O14" s="14" t="str">
@@ -1602,16 +1639,16 @@
         <v>11</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="C15" s="13" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="D15" s="13" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="E15" s="13" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="F15" s="11"/>
       <c r="G15" s="11"/>
@@ -1620,15 +1657,15 @@
       <c r="J15" s="11"/>
       <c r="K15" s="11"/>
       <c r="L15" s="14" t="str">
-        <f aca="false">IF(F15="","",4*F15-(4*G15+H15)-4*F15*Assumptions!$B$5)</f>
+        <f aca="false">IF(F15="","",4*F15-(4*G15+H15)/Assumptions!$B$6-4*F15*Assumptions!$B$7)</f>
         <v/>
       </c>
       <c r="M15" s="14" t="str">
-        <f aca="false">IF(F15="","",(Assumptions!$B$6+Assumptions!$B$7)*F15-((Assumptions!$B$6+Assumptions!$B$7)*G15+I15)-Assumptions!$B$7*K15-(Assumptions!$B$6+Assumptions!$B$7)*F15*Assumptions!$B$5)</f>
+        <f aca="false">IF(F15="","",(Assumptions!$B$8+Assumptions!$B$9)*F15-((Assumptions!$B$8+Assumptions!$B$9)*G15+I15)/Assumptions!$B$6-Assumptions!$B$9*K15-(Assumptions!$B$8+Assumptions!$B$9)*F15*Assumptions!$B$7)</f>
         <v/>
       </c>
       <c r="N15" s="14" t="str">
-        <f aca="false">IF(F15="","",(Assumptions!$B$8+Assumptions!$B$9)*F15-((Assumptions!$B$8+Assumptions!$B$9)*G15+J15)-Assumptions!$B$9*K15-(Assumptions!$B$8+Assumptions!$B$9)*F15*Assumptions!$B$5)</f>
+        <f aca="false">IF(F15="","",(Assumptions!$B$10+Assumptions!$B$11)*F15-((Assumptions!$B$10+Assumptions!$B$11)*G15+J15)/Assumptions!$B$6-Assumptions!$B$11*K15-(Assumptions!$B$10+Assumptions!$B$11)*F15*Assumptions!$B$7)</f>
         <v/>
       </c>
       <c r="O15" s="14" t="str">
@@ -1642,16 +1679,16 @@
         <v>12</v>
       </c>
       <c r="B16" s="13" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="C16" s="13" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="D16" s="13" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="E16" s="13" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="F16" s="11"/>
       <c r="G16" s="11"/>
@@ -1660,15 +1697,15 @@
       <c r="J16" s="11"/>
       <c r="K16" s="11"/>
       <c r="L16" s="14" t="str">
-        <f aca="false">IF(F16="","",4*F16-(4*G16+H16)-4*F16*Assumptions!$B$5)</f>
+        <f aca="false">IF(F16="","",4*F16-(4*G16+H16)/Assumptions!$B$6-4*F16*Assumptions!$B$7)</f>
         <v/>
       </c>
       <c r="M16" s="14" t="str">
-        <f aca="false">IF(F16="","",(Assumptions!$B$6+Assumptions!$B$7)*F16-((Assumptions!$B$6+Assumptions!$B$7)*G16+I16)-Assumptions!$B$7*K16-(Assumptions!$B$6+Assumptions!$B$7)*F16*Assumptions!$B$5)</f>
+        <f aca="false">IF(F16="","",(Assumptions!$B$8+Assumptions!$B$9)*F16-((Assumptions!$B$8+Assumptions!$B$9)*G16+I16)/Assumptions!$B$6-Assumptions!$B$9*K16-(Assumptions!$B$8+Assumptions!$B$9)*F16*Assumptions!$B$7)</f>
         <v/>
       </c>
       <c r="N16" s="14" t="str">
-        <f aca="false">IF(F16="","",(Assumptions!$B$8+Assumptions!$B$9)*F16-((Assumptions!$B$8+Assumptions!$B$9)*G16+J16)-Assumptions!$B$9*K16-(Assumptions!$B$8+Assumptions!$B$9)*F16*Assumptions!$B$5)</f>
+        <f aca="false">IF(F16="","",(Assumptions!$B$10+Assumptions!$B$11)*F16-((Assumptions!$B$10+Assumptions!$B$11)*G16+J16)/Assumptions!$B$6-Assumptions!$B$11*K16-(Assumptions!$B$10+Assumptions!$B$11)*F16*Assumptions!$B$7)</f>
         <v/>
       </c>
       <c r="O16" s="14" t="str">
@@ -1682,16 +1719,16 @@
         <v>13</v>
       </c>
       <c r="B17" s="13" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="C17" s="13" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="D17" s="13" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="E17" s="13" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="F17" s="11"/>
       <c r="G17" s="11"/>
@@ -1700,15 +1737,15 @@
       <c r="J17" s="11"/>
       <c r="K17" s="11"/>
       <c r="L17" s="14" t="str">
-        <f aca="false">IF(F17="","",4*F17-(4*G17+H17)-4*F17*Assumptions!$B$5)</f>
+        <f aca="false">IF(F17="","",4*F17-(4*G17+H17)/Assumptions!$B$6-4*F17*Assumptions!$B$7)</f>
         <v/>
       </c>
       <c r="M17" s="14" t="str">
-        <f aca="false">IF(F17="","",(Assumptions!$B$6+Assumptions!$B$7)*F17-((Assumptions!$B$6+Assumptions!$B$7)*G17+I17)-Assumptions!$B$7*K17-(Assumptions!$B$6+Assumptions!$B$7)*F17*Assumptions!$B$5)</f>
+        <f aca="false">IF(F17="","",(Assumptions!$B$8+Assumptions!$B$9)*F17-((Assumptions!$B$8+Assumptions!$B$9)*G17+I17)/Assumptions!$B$6-Assumptions!$B$9*K17-(Assumptions!$B$8+Assumptions!$B$9)*F17*Assumptions!$B$7)</f>
         <v/>
       </c>
       <c r="N17" s="14" t="str">
-        <f aca="false">IF(F17="","",(Assumptions!$B$8+Assumptions!$B$9)*F17-((Assumptions!$B$8+Assumptions!$B$9)*G17+J17)-Assumptions!$B$9*K17-(Assumptions!$B$8+Assumptions!$B$9)*F17*Assumptions!$B$5)</f>
+        <f aca="false">IF(F17="","",(Assumptions!$B$10+Assumptions!$B$11)*F17-((Assumptions!$B$10+Assumptions!$B$11)*G17+J17)/Assumptions!$B$6-Assumptions!$B$11*K17-(Assumptions!$B$10+Assumptions!$B$11)*F17*Assumptions!$B$7)</f>
         <v/>
       </c>
       <c r="O17" s="14" t="str">
@@ -1716,7 +1753,7 @@
         <v/>
       </c>
       <c r="P17" s="13" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1724,16 +1761,16 @@
         <v>14</v>
       </c>
       <c r="B18" s="13" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="C18" s="13" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="D18" s="13" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="E18" s="13" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="F18" s="11"/>
       <c r="G18" s="11"/>
@@ -1742,15 +1779,15 @@
       <c r="J18" s="11"/>
       <c r="K18" s="11"/>
       <c r="L18" s="14" t="str">
-        <f aca="false">IF(F18="","",4*F18-(4*G18+H18)-4*F18*Assumptions!$B$5)</f>
+        <f aca="false">IF(F18="","",4*F18-(4*G18+H18)/Assumptions!$B$6-4*F18*Assumptions!$B$7)</f>
         <v/>
       </c>
       <c r="M18" s="14" t="str">
-        <f aca="false">IF(F18="","",(Assumptions!$B$6+Assumptions!$B$7)*F18-((Assumptions!$B$6+Assumptions!$B$7)*G18+I18)-Assumptions!$B$7*K18-(Assumptions!$B$6+Assumptions!$B$7)*F18*Assumptions!$B$5)</f>
+        <f aca="false">IF(F18="","",(Assumptions!$B$8+Assumptions!$B$9)*F18-((Assumptions!$B$8+Assumptions!$B$9)*G18+I18)/Assumptions!$B$6-Assumptions!$B$9*K18-(Assumptions!$B$8+Assumptions!$B$9)*F18*Assumptions!$B$7)</f>
         <v/>
       </c>
       <c r="N18" s="14" t="str">
-        <f aca="false">IF(F18="","",(Assumptions!$B$8+Assumptions!$B$9)*F18-((Assumptions!$B$8+Assumptions!$B$9)*G18+J18)-Assumptions!$B$9*K18-(Assumptions!$B$8+Assumptions!$B$9)*F18*Assumptions!$B$5)</f>
+        <f aca="false">IF(F18="","",(Assumptions!$B$10+Assumptions!$B$11)*F18-((Assumptions!$B$10+Assumptions!$B$11)*G18+J18)/Assumptions!$B$6-Assumptions!$B$11*K18-(Assumptions!$B$10+Assumptions!$B$11)*F18*Assumptions!$B$7)</f>
         <v/>
       </c>
       <c r="O18" s="14" t="str">
@@ -1758,7 +1795,7 @@
         <v/>
       </c>
       <c r="P18" s="13" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1766,16 +1803,16 @@
         <v>15</v>
       </c>
       <c r="B19" s="13" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="C19" s="13" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="D19" s="13" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="E19" s="13" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="F19" s="11"/>
       <c r="G19" s="11"/>
@@ -1784,15 +1821,15 @@
       <c r="J19" s="11"/>
       <c r="K19" s="11"/>
       <c r="L19" s="14" t="str">
-        <f aca="false">IF(F19="","",4*F19-(4*G19+H19)-4*F19*Assumptions!$B$5)</f>
+        <f aca="false">IF(F19="","",4*F19-(4*G19+H19)/Assumptions!$B$6-4*F19*Assumptions!$B$7)</f>
         <v/>
       </c>
       <c r="M19" s="14" t="str">
-        <f aca="false">IF(F19="","",(Assumptions!$B$6+Assumptions!$B$7)*F19-((Assumptions!$B$6+Assumptions!$B$7)*G19+I19)-Assumptions!$B$7*K19-(Assumptions!$B$6+Assumptions!$B$7)*F19*Assumptions!$B$5)</f>
+        <f aca="false">IF(F19="","",(Assumptions!$B$8+Assumptions!$B$9)*F19-((Assumptions!$B$8+Assumptions!$B$9)*G19+I19)/Assumptions!$B$6-Assumptions!$B$9*K19-(Assumptions!$B$8+Assumptions!$B$9)*F19*Assumptions!$B$7)</f>
         <v/>
       </c>
       <c r="N19" s="14" t="str">
-        <f aca="false">IF(F19="","",(Assumptions!$B$8+Assumptions!$B$9)*F19-((Assumptions!$B$8+Assumptions!$B$9)*G19+J19)-Assumptions!$B$9*K19-(Assumptions!$B$8+Assumptions!$B$9)*F19*Assumptions!$B$5)</f>
+        <f aca="false">IF(F19="","",(Assumptions!$B$10+Assumptions!$B$11)*F19-((Assumptions!$B$10+Assumptions!$B$11)*G19+J19)/Assumptions!$B$6-Assumptions!$B$11*K19-(Assumptions!$B$10+Assumptions!$B$11)*F19*Assumptions!$B$7)</f>
         <v/>
       </c>
       <c r="O19" s="14" t="str">
@@ -1806,16 +1843,16 @@
         <v>16</v>
       </c>
       <c r="B20" s="13" t="s">
+        <v>90</v>
+      </c>
+      <c r="C20" s="13" t="s">
         <v>85</v>
       </c>
-      <c r="C20" s="13" t="s">
-        <v>80</v>
-      </c>
       <c r="D20" s="13" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="E20" s="13" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="F20" s="11"/>
       <c r="G20" s="11"/>
@@ -1824,15 +1861,15 @@
       <c r="J20" s="11"/>
       <c r="K20" s="11"/>
       <c r="L20" s="14" t="str">
-        <f aca="false">IF(F20="","",4*F20-(4*G20+H20)-4*F20*Assumptions!$B$5)</f>
+        <f aca="false">IF(F20="","",4*F20-(4*G20+H20)/Assumptions!$B$6-4*F20*Assumptions!$B$7)</f>
         <v/>
       </c>
       <c r="M20" s="14" t="str">
-        <f aca="false">IF(F20="","",(Assumptions!$B$6+Assumptions!$B$7)*F20-((Assumptions!$B$6+Assumptions!$B$7)*G20+I20)-Assumptions!$B$7*K20-(Assumptions!$B$6+Assumptions!$B$7)*F20*Assumptions!$B$5)</f>
+        <f aca="false">IF(F20="","",(Assumptions!$B$8+Assumptions!$B$9)*F20-((Assumptions!$B$8+Assumptions!$B$9)*G20+I20)/Assumptions!$B$6-Assumptions!$B$9*K20-(Assumptions!$B$8+Assumptions!$B$9)*F20*Assumptions!$B$7)</f>
         <v/>
       </c>
       <c r="N20" s="14" t="str">
-        <f aca="false">IF(F20="","",(Assumptions!$B$8+Assumptions!$B$9)*F20-((Assumptions!$B$8+Assumptions!$B$9)*G20+J20)-Assumptions!$B$9*K20-(Assumptions!$B$8+Assumptions!$B$9)*F20*Assumptions!$B$5)</f>
+        <f aca="false">IF(F20="","",(Assumptions!$B$10+Assumptions!$B$11)*F20-((Assumptions!$B$10+Assumptions!$B$11)*G20+J20)/Assumptions!$B$6-Assumptions!$B$11*K20-(Assumptions!$B$10+Assumptions!$B$11)*F20*Assumptions!$B$7)</f>
         <v/>
       </c>
       <c r="O20" s="14" t="str">
@@ -1875,111 +1912,111 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="9" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="F3" s="9" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="G3" s="9" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="H3" s="9" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="I3" s="9" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="J3" s="9" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="K3" s="9" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="L3" s="9" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="M3" s="9" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="N3" s="9" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="O3" s="9" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="P3" s="9" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="Q3" s="9" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="R3" s="9" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="10" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="E4" s="11" t="n">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="F4" s="11" t="n">
         <v>900</v>
       </c>
       <c r="G4" s="11" t="n">
-        <v>180</v>
+        <v>9900</v>
       </c>
       <c r="H4" s="11" t="n">
-        <v>700</v>
+        <v>38500</v>
       </c>
       <c r="I4" s="11" t="n">
-        <v>600</v>
+        <v>33000</v>
       </c>
       <c r="J4" s="11" t="n">
-        <v>120</v>
+        <v>6600</v>
       </c>
       <c r="K4" s="11" t="n">
-        <v>160</v>
+        <v>8800</v>
       </c>
       <c r="L4" s="11" t="n">
-        <v>200</v>
+        <v>11000</v>
       </c>
       <c r="M4" s="11" t="n">
         <v>60</v>
       </c>
       <c r="N4" s="12" t="n">
-        <f aca="false">IF(F4="","",4*F4-(4*G4+2*H4+J4)-4*F4*Assumptions!$B$5)</f>
+        <f aca="false">IF(F4="","",4*F4-(4*G4+2*H4+J4)/Assumptions!$B$6-4*F4*Assumptions!$B$7)</f>
         <v>1252</v>
       </c>
       <c r="O4" s="12" t="n">
-        <f aca="false">IF(F4="","",4*F4-(4*G4+1*H4+2*I4+J4)-4*F4*Assumptions!$B$5)</f>
+        <f aca="false">IF(F4="","",4*F4-(4*G4+1*H4+2*I4+J4)/Assumptions!$B$6-4*F4*Assumptions!$B$7)</f>
         <v>752</v>
       </c>
       <c r="P4" s="12" t="n">
@@ -1991,7 +2028,7 @@
         <v>OK</v>
       </c>
       <c r="R4" s="10" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1999,13 +2036,13 @@
         <v>17</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="C5" s="13" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="D5" s="13" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="E5" s="11"/>
       <c r="F5" s="11"/>
@@ -2017,11 +2054,11 @@
       <c r="L5" s="11"/>
       <c r="M5" s="11"/>
       <c r="N5" s="14" t="str">
-        <f aca="false">IF(F5="","",4*F5-(4*G5+2*H5+J5)-4*F5*Assumptions!$B$5)</f>
+        <f aca="false">IF(F5="","",4*F5-(4*G5+2*H5+J5)/Assumptions!$B$6-4*F5*Assumptions!$B$7)</f>
         <v/>
       </c>
       <c r="O5" s="14" t="str">
-        <f aca="false">IF(F5="","",4*F5-(4*G5+1*H5+2*I5+J5)-4*F5*Assumptions!$B$5)</f>
+        <f aca="false">IF(F5="","",4*F5-(4*G5+1*H5+2*I5+J5)/Assumptions!$B$6-4*F5*Assumptions!$B$7)</f>
         <v/>
       </c>
       <c r="P5" s="14" t="str">
@@ -2039,13 +2076,13 @@
         <v>18</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="D6" s="13" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="E6" s="11"/>
       <c r="F6" s="11"/>
@@ -2057,11 +2094,11 @@
       <c r="L6" s="11"/>
       <c r="M6" s="11"/>
       <c r="N6" s="14" t="str">
-        <f aca="false">IF(F6="","",4*F6-(4*G6+2*H6+J6)-4*F6*Assumptions!$B$5)</f>
+        <f aca="false">IF(F6="","",4*F6-(4*G6+2*H6+J6)/Assumptions!$B$6-4*F6*Assumptions!$B$7)</f>
         <v/>
       </c>
       <c r="O6" s="14" t="str">
-        <f aca="false">IF(F6="","",4*F6-(4*G6+1*H6+2*I6+J6)-4*F6*Assumptions!$B$5)</f>
+        <f aca="false">IF(F6="","",4*F6-(4*G6+1*H6+2*I6+J6)/Assumptions!$B$6-4*F6*Assumptions!$B$7)</f>
         <v/>
       </c>
       <c r="P6" s="14" t="str">
@@ -2079,13 +2116,13 @@
         <v>19</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="C7" s="13" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="D7" s="13" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="E7" s="11"/>
       <c r="F7" s="11"/>
@@ -2097,11 +2134,11 @@
       <c r="L7" s="11"/>
       <c r="M7" s="11"/>
       <c r="N7" s="14" t="str">
-        <f aca="false">IF(F7="","",4*F7-(4*G7+2*H7+J7)-4*F7*Assumptions!$B$5)</f>
+        <f aca="false">IF(F7="","",4*F7-(4*G7+2*H7+J7)/Assumptions!$B$6-4*F7*Assumptions!$B$7)</f>
         <v/>
       </c>
       <c r="O7" s="14" t="str">
-        <f aca="false">IF(F7="","",4*F7-(4*G7+1*H7+2*I7+J7)-4*F7*Assumptions!$B$5)</f>
+        <f aca="false">IF(F7="","",4*F7-(4*G7+1*H7+2*I7+J7)/Assumptions!$B$6-4*F7*Assumptions!$B$7)</f>
         <v/>
       </c>
       <c r="P7" s="14" t="str">
@@ -2119,13 +2156,13 @@
         <v>20</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="C8" s="13" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="D8" s="13" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="E8" s="11"/>
       <c r="F8" s="11"/>
@@ -2137,11 +2174,11 @@
       <c r="L8" s="11"/>
       <c r="M8" s="11"/>
       <c r="N8" s="14" t="str">
-        <f aca="false">IF(F8="","",4*F8-(4*G8+2*H8+J8)-4*F8*Assumptions!$B$5)</f>
+        <f aca="false">IF(F8="","",4*F8-(4*G8+2*H8+J8)/Assumptions!$B$6-4*F8*Assumptions!$B$7)</f>
         <v/>
       </c>
       <c r="O8" s="14" t="str">
-        <f aca="false">IF(F8="","",4*F8-(4*G8+1*H8+2*I8+J8)-4*F8*Assumptions!$B$5)</f>
+        <f aca="false">IF(F8="","",4*F8-(4*G8+1*H8+2*I8+J8)/Assumptions!$B$6-4*F8*Assumptions!$B$7)</f>
         <v/>
       </c>
       <c r="P8" s="14" t="str">
@@ -2159,13 +2196,13 @@
         <v>21</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="D9" s="13" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="E9" s="11"/>
       <c r="F9" s="11"/>
@@ -2177,11 +2214,11 @@
       <c r="L9" s="11"/>
       <c r="M9" s="11"/>
       <c r="N9" s="14" t="str">
-        <f aca="false">IF(F9="","",4*F9-(4*G9+2*H9+J9)-4*F9*Assumptions!$B$5)</f>
+        <f aca="false">IF(F9="","",4*F9-(4*G9+2*H9+J9)/Assumptions!$B$6-4*F9*Assumptions!$B$7)</f>
         <v/>
       </c>
       <c r="O9" s="14" t="str">
-        <f aca="false">IF(F9="","",4*F9-(4*G9+1*H9+2*I9+J9)-4*F9*Assumptions!$B$5)</f>
+        <f aca="false">IF(F9="","",4*F9-(4*G9+1*H9+2*I9+J9)/Assumptions!$B$6-4*F9*Assumptions!$B$7)</f>
         <v/>
       </c>
       <c r="P9" s="14" t="str">
@@ -2193,7 +2230,7 @@
         <v/>
       </c>
       <c r="R9" s="13" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
     </row>
   </sheetData>
@@ -2221,41 +2258,41 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="15" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="B4" s="15" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="C4" s="15" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="D4" s="15" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="E4" s="15" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="F4" s="15" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="G4" s="15" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="H4" s="15" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="I4" s="15" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2263,7 +2300,7 @@
         <v>1</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="C5" s="16"/>
       <c r="D5" s="16"/>
@@ -2278,7 +2315,7 @@
         <v>2</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="C6" s="16"/>
       <c r="D6" s="16"/>
@@ -2293,7 +2330,7 @@
         <v>3</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="C7" s="16"/>
       <c r="D7" s="16"/>
@@ -2308,7 +2345,7 @@
         <v>4</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="C8" s="16"/>
       <c r="D8" s="16"/>
@@ -2323,7 +2360,7 @@
         <v>5</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="C9" s="16"/>
       <c r="D9" s="16"/>
@@ -2338,7 +2375,7 @@
         <v>6</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="C10" s="16"/>
       <c r="D10" s="16"/>
@@ -2353,7 +2390,7 @@
         <v>7</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="C11" s="16"/>
       <c r="D11" s="16"/>
@@ -2368,7 +2405,7 @@
         <v>8</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="C12" s="16"/>
       <c r="D12" s="16"/>
@@ -2383,7 +2420,7 @@
         <v>9</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="C13" s="16"/>
       <c r="D13" s="16"/>
@@ -2398,7 +2435,7 @@
         <v>10</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="C14" s="16"/>
       <c r="D14" s="16"/>
@@ -2413,7 +2450,7 @@
         <v>11</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="C15" s="16"/>
       <c r="D15" s="16"/>
@@ -2428,7 +2465,7 @@
         <v>12</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="C16" s="16"/>
       <c r="D16" s="16"/>
@@ -2443,7 +2480,7 @@
         <v>13</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="C17" s="16"/>
       <c r="D17" s="16"/>
@@ -2458,7 +2495,7 @@
         <v>14</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="C18" s="16"/>
       <c r="D18" s="16"/>
@@ -2473,7 +2510,7 @@
         <v>15</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="C19" s="16"/>
       <c r="D19" s="16"/>
@@ -2488,7 +2525,7 @@
         <v>16</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="C20" s="16"/>
       <c r="D20" s="16"/>
@@ -2503,7 +2540,7 @@
         <v>17</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="C21" s="16"/>
       <c r="D21" s="16"/>
@@ -2518,7 +2555,7 @@
         <v>18</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="C22" s="16"/>
       <c r="D22" s="16"/>
@@ -2533,7 +2570,7 @@
         <v>19</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="C23" s="16"/>
       <c r="D23" s="16"/>
@@ -2548,7 +2585,7 @@
         <v>20</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="C24" s="16"/>
       <c r="D24" s="16"/>
@@ -2563,7 +2600,7 @@
         <v>21</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="C25" s="16"/>
       <c r="D25" s="16"/>

</xml_diff>